<commit_message>
update for phase 4
</commit_message>
<xml_diff>
--- a/tester/fixtures/phase4/contrast_vectors.xlsx
+++ b/tester/fixtures/phase4/contrast_vectors.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="16">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -102,8 +102,23 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4" tint="-0.5"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="8" tint="-0.5"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9" tint="-0.5"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -138,6 +153,12 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF757575"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -151,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -171,6 +192,9 @@
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -294,10 +318,10 @@
         <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="050505"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="010101"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="0000FF"/>
@@ -500,7 +524,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,6 +552,27 @@
       <c r="A7" s="11" t="inlineStr">
         <is>
           <t>dk1 tint 0.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>accent1 tint -0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>050505 tint -0.5 on 757575</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>010101 tint -0.5</t>
         </is>
       </c>
     </row>

</xml_diff>